<commit_message>
Update configs, add new scripts, and refresh scour output
- Modified: app_config.json, debug_analysis.py, guide_mappings.json,
  networking_terms.json, requirements.txt, sidebar_app.py,
  sidebar_resolve_bug_page.py, testresults-analysisAmel.xlsx
- Updated scour_output (draft_concept_mappings, gap_report, raw_results, summary)
- Added: downloadbooks.py, fetch_bug.py, guide_mappings.json.bak,
  merge_scour_concepts.py, product_keywords.json
</commit_message>
<xml_diff>
--- a/testresults-analysisAmel.xlsx
+++ b/testresults-analysisAmel.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amabdulr/Library/CloudStorage/OneDrive-Cisco/Lair/Python/January/Denver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5E1861D-B436-814C-9152-5633FCE425AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD0B8F9-CCE4-EA47-8AFC-E60EA47CABCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28380" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2600" yWindow="1040" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="145">
   <si>
     <t>Timestamp</t>
   </si>
@@ -305,9 +318,6 @@
   </si>
   <si>
     <t>2026-02-12 11:15:23</t>
-  </si>
-  <si>
-    <t>699949022</t>
   </si>
   <si>
     <t>### Location Recommendations
@@ -401,9 +411,6 @@
     <t>2026-02-12 11:26:35</t>
   </si>
   <si>
-    <t>699939784</t>
-  </si>
-  <si>
     <t>Based on the information retrieved from the selected guides, here are the relevant documentation locations and content recommendations for the issue related to the "Configuration-db: System and/or Neo4j databases do not have the required member count" error during the Cisco SD-WAN upgrade:
 ### Location Recommendations
 1. **Document name:** sdwan-xe-gs-book.pdf
@@ -1124,42 +1131,9 @@
     <t>2026-02-13 21:05:00</t>
   </si>
   <si>
-    <t>partho</t>
-  </si>
-  <si>
     <t>CSCws43449</t>
   </si>
   <si>
-    <t>### Location Recommendations
-1. **Document name:** systems-interfaces-book-xe-sdwan.pdf
-   - **Part/Section hierarchy:** CHAPTER 33 Cisco Catalyst SD-WAN EtherChannel
-   - **Page number:** Page 825
-   - **Actual content location indicator:** "The number of supported port channels differs based on the specific device model."
-   - **Detailed reasoning:** This section discusses the variability in the number of supported port channels and member interfaces for EtherChannel, which directly relates to the need for specific information on the maximum number of supported EtherChannel member links for each hardware device.
-2. **Document name:** systems-interfaces-book-xe-sdwan.pdf
-   - **Part/Section hierarchy:** CHAPTER 33 Cisco Catalyst SD-WAN EtherChannel
-   - **Page number:** Page 837
-   - **Actual content location indicator:** "The maximum number of port channel interfaces that a device can support varies, depending on the particular model of the device."
-   - **Detailed reasoning:** This section highlights the restrictions and variability in the maximum number of port channel interfaces supported by different device models, which is pertinent to the issue of needing clear documentation on supported member links per hardware platform.
-3. **Document name:** systems-interfaces-book-xe-sdwan.pdf
-   - **Part/Section hierarchy:** CHAPTER 33 Cisco Catalyst SD-WAN EtherChannel
-   - **Page number:** Page 830
-   - **Actual content location indicator:** "The maximum number of port channel interfaces that a device can support varies, depending on the particular model of the device."
-   - **Detailed reasoning:** This section reiterates the variability in support for port channel interfaces across different device models, emphasizing the need for specific documentation on the maximum number of supported member links.
-### Documentation Content
-**Problem Summary:** The current documentation lacks specific details on the maximum number of supported EtherChannel member links for each hardware device model, leading to ambiguity and potential configuration issues.
-**Recommended Guide:** systems-interfaces-book-xe-sdwan.pdf
-**Documentation Strategy:** Provide detailed specifications for each hardware model regarding the maximum number of supported EtherChannel member links to ensure clear and precise configuration guidance.
-**Actual Documentation Content:**
-- **Behavior Explanation:** The number of supported EtherChannel member links can vary significantly depending on the specific hardware model. This variability can affect network configuration and performance if not properly documented and understood.
-- **Configuration Steps:**
-  1. Identify the specific hardware model in use.
-  2. Refer to the updated documentation section for the exact number of supported EtherChannel member links for that model.
-  3. Configure the EtherChannel accordingly, ensuring that the number of member links does not exceed the documented limit.
-- **Recommended Format:** This content should be documented as a configuration guide with specific model-based details to aid network engineers in setting up EtherChannels correctly.
-This documentation content aims to provide a clear understanding of the supported configurations for EtherChannels on various Cisco SD-WAN devices, ensuring that users can manage their network configurations effectively.</t>
-  </si>
-  <si>
     <t xml:space="preserve">ANALYZED </t>
   </si>
   <si>
@@ -1175,7 +1149,71 @@
     <t>Unclear comment</t>
   </si>
   <si>
+    <t>Executive Summary:
+The customer, Orange, experienced a critical issue on their Cisco Catalyst C8300-1N1S-6T Router managed via vManage (software version 20.12.4.1), where it was impossible to push a new security group policy. Although the stuck deployment task was cleared from the vManage GUI using the API clean command, attempts to deploy a new policy resulted in the error: "Policy group state validation error: A deployment for Policy Group [name of the policy] is in-progress. Please wait to complete." This blocked all migrations and network changes for the customer. The root cause was a residual deployment task in the Neo4j database that was not cleared by the API, requiring manual intervention at the database level. The issue was resolved by editing the Neo4j database entry for the stuck task from "Deploying" to "Deploy Failure," which allowed policy deployment to proceed and unblocked migrations.
+Steps to Reproduce:
+1. Initiate a security group policy deployment from vManage to a group of cEdge routers.
+2. Observe that the deployment task becomes stuck in "in_progress" state (visible via API: /dataservice/device/action/status/tasks).
+3. Attempt to clean the stuck task using the API endpoint: /dataservice/device/action/status/tasks/clean?processId=&lt;processId&gt;.
+4. Verify that no running tasks are visible in the vManage GUI.
+5. Attempt to push a new security group policy.
+6. Encounter the error: "Policy group state validation error: A deployment for Policy Group [name of the policy] is in-progress. Please wait to complete."
+7. Confirm that migrations and policy changes are blocked.
+Condition:
+- vManage is running on-premises, managing Cisco Catalyst C8300-1N1S-6T routers.
+- Software version: vManage 20.12.4.1.
+- The stuck deployment task is for a security policy group push to cEdge devices.
+- The API shows no running tasks after clean-up, but the Neo4j database still contains a task with status "in_progress" for processId "deploy_policy_group-5d19b44b-30ab-44c8-a192-305208e724be".
+- Admin tech and error screenshots confirm the persistent error.
+- All migrations for the customer are blocked due to this condition.
+Workarounds:
+- No effective workaround was available via the vManage GUI or API; the only temporary mitigation was to avoid further policy pushes until the database was manually corrected.
+- Manual intervention in the Neo4j database was required to resolve the issue.
+Procedure (Solution):
+1. Schedule a Webex session with the customer to access the vManage system.
+2. Obtain admin tech and error screenshots for analysis.
+3. Access the Neo4j database on the vManage server.
+4. Locate the stuck deployment task using the processId "deploy_policy_group-5d19b44b-30ab-44c8-a192-305208e724be".
+5. Execute Neo4j queries to change the task status from "Deploying" to "Deploy Failure". Example query:
+   ```
+   MATCH (n) WHERE n.processId = 'deploy_policy_group-5d19b44b-30ab-44c8-a192-305208e724be'
+   SET n.status = 'deploy_failure'
+   ```
+6. Verify that the change is reflected and no tasks are stuck in "in_progress" state.
+7. Attempt to push the security group policy again from vManage.
+8. Confirm successful deployment and unblock migrations.
+Root Cause:
+The root cause was a race condition or software defect where a deployment task for a policy group remained in the Neo4j database with a status of "in_progress" even after the API clean command was executed and the task was no longer visible in the vManage GUI. This residual database entry caused vManage to block any new policy group deployments, resulting in the error: "Policy group state validation error: A deployment for Policy Group [name of the policy] is in-progress. Please wait to complete." Technical indicators included:
+- API output showing the stuck task:
+  ```
+  {"runningTasks":[{"detailsURL":"/dataservice/device/action/status","scheduledAction":false,"userSessionUserName":"UA01317339T8","@rid":30573,"tenantName":"DefaultTenant","processId":"deploy_policy_group-5d19b44b-30ab-44c8-a192-305208e724be","userSessionIP":"10.248.35.61","name":"Deploy policy group to associated devices","tenantId":"default","action":"deploy_policy_group","startTime":1761149650791,"endTime":0,"status":"in_progress"}]}
+  ```
+- Error message in vManage GUI and logs:
+  ```
+  "Policy group state validation error: A deployment for Policy Group [name of the policy] is in-progress. Please wait to complete."
+  ```
+- Attempts to clean the task via API did not remove the Neo4j database entry.
+- Manual Neo4j intervention was required to update the task status, after which policy deployment succeeded.
+Affected Devices/Versions:
+- Cisco Catalyst C8300-1N1S-6T Router managed via vManage.
+- vManage software version 20.12.4.1.
+- All cEdge routers associated with the affected policy group.
+Bugs:
+No specific Cisco bug ID (CSC*) was referenced in the case notes. However, the behavior suggests a possible software defect or race condition in vManage task management and Neo4j database synchronization. If a bug is later identified, it should be referenced here.
+Fixed Versions, Patches:
+- Issue resolved by manual Neo4j database edit; no software patch was applied.
+- No fixed version or patch is currently documented for this specific issue. Customers experiencing similar symptoms should contact Cisco TAC for assistance until a permanent fix is released.
+---
+End Template</t>
+  </si>
+  <si>
     <t>RCA content</t>
+  </si>
+  <si>
+    <t>Correccted</t>
+  </si>
+  <si>
+    <t>amel</t>
   </si>
 </sst>
 </file>
@@ -1205,12 +1243,48 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -1252,7 +1326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1267,6 +1341,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1613,10 +1702,10 @@
         <v>10</v>
       </c>
       <c r="L1" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="78" customHeight="1" x14ac:dyDescent="0.2">
@@ -1654,71 +1743,74 @@
         <v>19</v>
       </c>
       <c r="L2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="10">
         <v>8</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="10">
         <v>6</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="11">
         <v>4</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="11">
         <v>5</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="11" t="s">
         <v>19</v>
+      </c>
+      <c r="N4" s="11">
+        <v>8000</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -1746,7 +1838,7 @@
       <c r="H5">
         <v>9</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="8" t="s">
         <v>37</v>
       </c>
       <c r="J5" t="s">
@@ -1756,73 +1848,73 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="192" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:14" s="8" customFormat="1" ht="192" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <v>5</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="8">
         <v>3</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="L6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="277" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="L6" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="6" customFormat="1" ht="277" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="6">
         <v>699968875</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="6">
         <v>9</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>9</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="6" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1839,11 +1931,11 @@
       <c r="D8" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8">
+        <v>699949022</v>
+      </c>
+      <c r="F8" t="s">
         <v>49</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
       </c>
       <c r="G8">
         <v>10</v>
@@ -1852,7 +1944,7 @@
         <v>9</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K8" t="s">
         <v>25</v>
@@ -1860,7 +1952,7 @@
     </row>
     <row r="9" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
@@ -1875,7 +1967,7 @@
         <v>699942528</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1884,19 +1976,24 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K9" t="s">
         <v>25</v>
       </c>
+      <c r="L9" t="s">
+        <v>143</v>
+      </c>
       <c r="M9" t="s">
-        <v>140</v>
-      </c>
-      <c r="N9" s="2"/>
+        <v>136</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
@@ -1911,7 +2008,7 @@
         <v>699939784</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -1920,18 +2017,21 @@
         <v>7</v>
       </c>
       <c r="I10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K10" t="s">
         <v>25</v>
       </c>
+      <c r="L10" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
@@ -1942,11 +2042,11 @@
       <c r="D11" t="s">
         <v>45</v>
       </c>
-      <c r="E11" t="s">
-        <v>56</v>
+      <c r="E11">
+        <v>699939784</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1955,7 +2055,7 @@
         <v>7</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K11" t="s">
         <v>25</v>
@@ -1963,22 +2063,22 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G12">
         <v>8</v>
@@ -1987,10 +2087,10 @@
         <v>9</v>
       </c>
       <c r="I12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K12" t="s">
         <v>25</v>
@@ -1998,22 +2098,22 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" t="s">
         <v>65</v>
       </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="E13" t="s">
         <v>66</v>
       </c>
-      <c r="D13" t="s">
+      <c r="F13" t="s">
         <v>67</v>
-      </c>
-      <c r="E13" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" t="s">
-        <v>69</v>
       </c>
       <c r="G13">
         <v>9</v>
@@ -2027,22 +2127,22 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s">
         <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G14">
         <v>5</v>
@@ -2051,10 +2151,10 @@
         <v>4</v>
       </c>
       <c r="I14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K14" t="s">
         <v>19</v>
@@ -2062,7 +2162,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
@@ -2071,13 +2171,13 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G15">
         <v>9</v>
@@ -2086,7 +2186,7 @@
         <v>10</v>
       </c>
       <c r="I15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K15" t="s">
         <v>25</v>
@@ -2094,7 +2194,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
@@ -2103,13 +2203,13 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G16">
         <v>8</v>
@@ -2118,7 +2218,7 @@
         <v>8</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K16" t="s">
         <v>25</v>
@@ -2126,7 +2226,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
@@ -2135,13 +2235,13 @@
         <v>13</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G17">
         <v>6</v>
@@ -2150,59 +2250,59 @@
         <v>8</v>
       </c>
       <c r="I17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="K17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="18" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="B18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18">
+      <c r="G18" s="14">
         <v>3</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="14">
         <v>7</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="14" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" t="s">
         <v>90</v>
       </c>
-      <c r="B19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>91</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" t="s">
         <v>92</v>
-      </c>
-      <c r="E19" t="s">
-        <v>93</v>
-      </c>
-      <c r="F19" t="s">
-        <v>94</v>
       </c>
       <c r="G19">
         <v>10</v>
@@ -2216,22 +2316,22 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" t="s">
         <v>95</v>
-      </c>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" t="s">
-        <v>92</v>
-      </c>
-      <c r="E20" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" t="s">
-        <v>97</v>
       </c>
       <c r="G20">
         <v>10</v>
@@ -2245,7 +2345,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
@@ -2257,7 +2357,7 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G21">
         <v>8</v>
@@ -2266,15 +2366,15 @@
         <v>9</v>
       </c>
       <c r="I21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
@@ -2286,7 +2386,7 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G22">
         <v>9</v>
@@ -2295,30 +2395,30 @@
         <v>8</v>
       </c>
       <c r="I22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J22" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" t="s">
         <v>105</v>
       </c>
-      <c r="B23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>106</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>107</v>
-      </c>
-      <c r="E23" t="s">
-        <v>108</v>
-      </c>
-      <c r="F23" t="s">
-        <v>109</v>
       </c>
       <c r="G23">
         <v>10</v>
@@ -2327,97 +2427,97 @@
         <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="K23" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="24" spans="1:14" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A24" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="B24" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="E24" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="D24" t="s">
+      <c r="F24" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="E24" t="s">
+      <c r="G24" s="12">
+        <v>2</v>
+      </c>
+      <c r="H24" s="12">
+        <v>1</v>
+      </c>
+      <c r="I24" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="K24" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A25" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="G24">
+      <c r="B25" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="G25" s="12">
         <v>2</v>
       </c>
-      <c r="H24">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="K24" t="s">
-        <v>19</v>
-      </c>
-      <c r="N24" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>117</v>
-      </c>
-      <c r="B25" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>113</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="H25" s="12">
+        <v>3</v>
+      </c>
+      <c r="I25" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="F25" t="s">
-        <v>119</v>
-      </c>
-      <c r="G25">
-        <v>2</v>
-      </c>
-      <c r="H25">
-        <v>3</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="K25" t="s">
+      <c r="K25" s="12" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>120</v>
+      </c>
+      <c r="E26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" t="s">
         <v>121</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" t="s">
-        <v>122</v>
-      </c>
-      <c r="E26" t="s">
-        <v>108</v>
-      </c>
-      <c r="F26" t="s">
-        <v>123</v>
       </c>
       <c r="G26">
         <v>10</v>
@@ -2426,7 +2526,7 @@
         <v>10</v>
       </c>
       <c r="I26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K26" t="s">
         <v>25</v>
@@ -2434,19 +2534,19 @@
     </row>
     <row r="27" spans="1:14" ht="197" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F27" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G27">
         <v>10</v>
@@ -2455,7 +2555,7 @@
         <v>10</v>
       </c>
       <c r="I27" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K27" t="s">
         <v>25</v>
@@ -2463,19 +2563,19 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>120</v>
+      </c>
+      <c r="E28" t="s">
+        <v>127</v>
+      </c>
+      <c r="F28" t="s">
         <v>128</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" t="s">
-        <v>122</v>
-      </c>
-      <c r="E28" t="s">
-        <v>129</v>
-      </c>
-      <c r="F28" t="s">
-        <v>130</v>
       </c>
       <c r="G28">
         <v>10</v>
@@ -2484,7 +2584,7 @@
         <v>10</v>
       </c>
       <c r="I28" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K28" t="s">
         <v>25</v>
@@ -2492,19 +2592,19 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" t="s">
+        <v>131</v>
+      </c>
+      <c r="F29" t="s">
         <v>132</v>
-      </c>
-      <c r="B29" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" t="s">
-        <v>122</v>
-      </c>
-      <c r="E29" t="s">
-        <v>133</v>
-      </c>
-      <c r="F29" t="s">
-        <v>134</v>
       </c>
       <c r="G29">
         <v>10</v>
@@ -2513,38 +2613,36 @@
         <v>10</v>
       </c>
       <c r="I29" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J29" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>136</v>
-      </c>
-      <c r="B30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" t="s">
-        <v>137</v>
-      </c>
-      <c r="E30" t="s">
-        <v>138</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G30">
+    <row r="30" spans="1:14" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F30" s="13"/>
+      <c r="G30" s="12">
         <v>7</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="12">
         <v>6</v>
       </c>
-      <c r="K30" t="s">
+      <c r="K30" s="12" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2553,6 +2651,7 @@
     <hyperlink ref="I11" r:id="rId1" location="Cisco_Concept.dita_e8549172-4a20-469d-8d62-e4a2d3b19187 - this is the right guide and section. The issue was about Upgrading the S/w image, but the location identified was SD-WAN manager cluster in Getting Started guide which is not correct.  The content suggestion was reasonable good. " display="https://www.cisco.com/c/en/us/td/docs/routers/sdwan/configuration/Monitor-And-Maintain/monitor-maintain-book/maintain.html#Cisco_Concept.dita_e8549172-4a20-469d-8d62-e4a2d3b19187 - this is the right guide and section. The issue was about Upgrading the S/w image, but the location identified was SD-WAN manager cluster in Getting Started guide which is not correct.  The content suggestion was reasonable good. " xr:uid="{063C14FF-205C-9E4D-8F96-2CAF8B196404}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter>
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Cisco Confidential</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Add SD-WAN download scripts, chapter extraction, and enriched document inventory
- Add downloadbooks_landing.py for downloading SD-WAN PDFs from Cisco
- Add downloadbooks_iot_collection.py for IoT doc downloads
- Add extract_chapters.py to scrape chapter metadata from book pages
- Update document_inventory.json with chapter data (307 chapters across 28 books)
- Update sidebar_bulk_analysis_page.py
- Remove old downloadbooks.py
</commit_message>
<xml_diff>
--- a/testresults-analysisAmel.xlsx
+++ b/testresults-analysisAmel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amabdulr/Library/CloudStorage/OneDrive-Cisco/Lair/Python/January/Denver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD0B8F9-CCE4-EA47-8AFC-E60EA47CABCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344FEA09-CC10-D447-8048-4A1DB5A888D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2600" yWindow="1040" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2060" yWindow="680" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="147">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1132,12 +1132,6 @@
   </si>
   <si>
     <t>CSCws43449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANALYZED </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analhyzed. </t>
   </si>
   <si>
     <t>comments fro tester</t>
@@ -1214,6 +1208,92 @@
   </si>
   <si>
     <t>amel</t>
+  </si>
+  <si>
+    <t>MAILED</t>
+  </si>
+  <si>
+    <t>Executive Summary:
+The customer attempted to upgrade their Cisco SDWAN vManage controller (vmanage-293139987.sdwan.cisco.com) from version 20.15.4 to 20.18.1 in a Cisco Cloud Hosted environment. The upgrade failed during the GUI pre-checks due to a "Configuration-db: System and/or Neo4j databases do not have the required member count" error. This prevented the upgrade from proceeding and caused delays in updating the SDWAN management infrastructure. The issue was traced to Cisco bug CSCwm11883, which blocks GUI upgrades when database member counts do not meet expected thresholds. The upgrade was successfully completed using a CLI workaround. Secondary issues included vSmart controllers losing control connections and certificates post-upgrade, requiring re-enrollment and static IPv6 assignment to restore full functionality.
+Steps to Reproduce:
+1. Initiate upgrade of vManage from version 20.15.4 to 20.18.1 via the vManage GUI.
+2. Observe pre-check failures, specifically:
+   - Error: "Failed: Configuration-db: System and/or Neo4j databases do not have the required member count"
+3. Attempt to proceed with upgrade; GUI blocks further progress.
+4. Consider forcing activation via CLI.
+5. If CLI workaround is used, upgrade completes successfully.
+6. Post-upgrade, attempt to upgrade vSmart controllers.
+7. vSmart upgrade fails/rolls back, vSmart loses control connection and certificate.
+8. vBond controllers experience intermittent loss of connectivity and IPv6 address assignment.
+9. Re-enroll vSmart and assign static IPv6 to vBond to restore control connections.
+Condition:
+- Cisco Cloud Hosted SDWAN environment.
+- Single-node vManage (vmanage-293139987.sdwan.cisco.com), two vBonds, two vSmarts.
+- Upgrade path: vManage 20.15.4 → 20.18.1.
+- Pre-checks during GUI upgrade require Configuration-db and Neo4j databases to meet specific member count requirements.
+- Known defect (CSCwm11883) causes pre-checks to fail in certain single-node/cloud deployments.
+- vSmart controllers running on AWS, subject to cloud network reachability and certificate synchronization.
+- vBond controllers rely on DHCP for IPv6; loss of DHCP or network flapping can impact control connections.
+Workarounds:
+- Upgrade vManage using CLI commands instead of GUI:
+  - `request software install &lt;VERSION&gt;`
+  - `request software activate &lt;VERSION&gt;`
+- Collect configuration-db backup before upgrade:
+  - `request nms configuration-db backup path [file_name_configdb]`
+- For vSmart/vBond certificate or connectivity issues:
+  - Re-enroll affected controllers via vManage GUI.
+  - Assign static IPv6 addresses to vBond controllers if DHCP fails.
+  - Bounce VPN 0 transport interfaces if control connections do not restore automatically.
+Procedure (Solution):
+1. Backup the configuration-db:
+   ```
+   request nms configuration-db backup path /home/admin/configdb-backup-20251022
+   ```
+2. Install and activate the new software version via CLI:
+   ```
+   request software install 20.18.1
+   request software activate 20.18.1
+   ```
+3. Monitor upgrade progress and system logs for errors.
+4. If vSmart controllers fail to upgrade or lose control connections:
+   - Remove affected vSmart from vManage via GUI.
+   - Re-add vSmart, allowing auto-installation of certificate.
+   - Push device template to vSmart.
+   - Verify control connections and certificate status.
+5. If vBond controllers lose IPv6 connectivity:
+   - Assign static IPv6 addresses via device template or CLI.
+   - Verify control connections to vSmart and vManage.
+6. Validate all controllers and management nodes are operational post-upgrade.
+Root Cause:
+- The primary root cause of the vManage upgrade failure was the GUI pre-check logic enforcing Configuration-db and Neo4j database member count requirements, as described in Cisco bug CSCwm11883. In single-node or certain cloud-hosted deployments, these checks may incorrectly fail, blocking GUI upgrades even when the system is otherwise healthy.
+- Technical indicators:
+  - GUI error: "Failed: Configuration-db: System and/or Neo4j databases do not have the required member count"
+  - Admin-tech logs (1.1.1.4-vmanage-0-20251022-132030-admin-tech.tar.gz) confirmed single-node deployment and database status.
+- Secondary root cause for vSmart/vBond issues:
+  - Repeated upgrade attempts and rollbacks led to certificate corruption and loss of control connections.
+  - vBond controllers lost IPv6 addresses due to DHCP failure or AWS network flapping, which prevented proper control plane establishment.
+  - vSmart lost its certificate, indicated by "ERR_MY_CERT_REJ_BY_SERV" and CRTREJSER errors in vManage logs.
+- Resolution required re-enrollment of vSmart and static IPv6 assignment to vBond.
+Affected Devices/Versions:
+- vManage: vmanage-293139987.sdwan.cisco.com (Cisco Cloud Hosted), upgrading from 20.15.4 to 20.18.1.
+- vSmart controllers: AWS-hosted, affected during upgrade/rollback.
+- vBond controllers: AWS-hosted, affected by IPv6/DHCP issues.
+- All devices in the Cisco Cloud Hosted SDWAN environment running the above versions.
+Bugs:
+- CSCwm11883: "Show checks on vManage - better error messages for database member count issues"
+  - Description: GUI upgrade fails due to incorrect database member count checks in single-node/cloud deployments.
+  - Workaround: Use CLI upgrade method.
+Fixed Versions, Patches:
+- The issue with GUI upgrade checks is addressed in future vManage releases (post-20.18.1) with improved error messaging and logic for database member count validation.
+- For current deployments, use CLI upgrade as a workaround per CSCwm11883.
+- No additional patches required for certificate/control connection issues; resolution is procedural (re-enrollment, static IPv6 assignment).
+---</t>
+  </si>
+  <si>
+    <t>IN TOP THREE&gt; BUT NOT CHOSEN</t>
+  </si>
+  <si>
+    <t>. Comment from Amel: the location redocumentations still indicate Introduction. However the Documentation Content has chosen the Prefix, Configuration Group location</t>
   </si>
 </sst>
 </file>
@@ -1334,7 +1414,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1356,6 +1435,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1701,11 +1781,11 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>142</v>
+      <c r="L1" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="78" customHeight="1" x14ac:dyDescent="0.2">
@@ -1743,73 +1823,73 @@
         <v>19</v>
       </c>
       <c r="L2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="B3" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>8</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>6</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>4</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>5</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="J4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="K4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="11">
+      <c r="N4" s="10">
         <v>8000</v>
       </c>
     </row>
@@ -1838,7 +1918,7 @@
       <c r="H5">
         <v>9</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>37</v>
       </c>
       <c r="J5" t="s">
@@ -1848,150 +1928,150 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="8" customFormat="1" ht="192" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:14" s="7" customFormat="1" ht="192" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="B6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>5</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>3</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L6" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" s="6" customFormat="1" ht="277" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="L6" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="11" customFormat="1" ht="277" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="B7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="11">
         <v>699968875</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="11">
         <v>9</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="11">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="11">
         <v>699949022</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="11">
         <v>10</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="11">
         <v>9</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="9" spans="1:14" s="11" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="11">
         <v>699942528</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="11">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="11">
         <v>5</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="M9" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="M9" t="s">
-        <v>136</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N9" s="12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -2026,39 +2106,45 @@
         <v>25</v>
       </c>
       <c r="L10" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+        <v>141</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" s="5" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="5">
         <v>699939784</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="5">
         <v>1</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="5">
         <v>7</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="5" t="s">
         <v>25</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -2256,32 +2342,32 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:14" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="14" t="s">
+      <c r="B18" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="13">
         <v>3</v>
       </c>
-      <c r="H18" s="14">
+      <c r="H18" s="13">
         <v>7</v>
       </c>
-      <c r="K18" s="14" t="s">
+      <c r="K18" s="13" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2436,70 +2522,70 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
+    <row r="24" spans="1:14" s="11" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="12" t="s">
+      <c r="B24" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="F24" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="G24" s="12">
+      <c r="G24" s="11">
         <v>2</v>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="11">
         <v>1</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="K24" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="N24" s="12" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
+      <c r="N24" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" s="11" customFormat="1" ht="380" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B25" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="B25" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="G25" s="12">
+      <c r="G25" s="11">
         <v>2</v>
       </c>
-      <c r="H25" s="12">
+      <c r="H25" s="11">
         <v>3</v>
       </c>
-      <c r="I25" s="13" t="s">
+      <c r="I25" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="K25" s="12" t="s">
+      <c r="K25" s="11" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2622,27 +2708,27 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="12" t="s">
+    <row r="30" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="B30" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E30" s="12" t="s">
+      <c r="B30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E30" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="F30" s="13"/>
-      <c r="G30" s="12">
+      <c r="F30" s="12"/>
+      <c r="G30" s="11">
         <v>7</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="11">
         <v>6</v>
       </c>
-      <c r="K30" s="12" t="s">
+      <c r="K30" s="11" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>